<commit_message>
Mise à jour du site depuis l'usine
</commit_message>
<xml_diff>
--- a/assets/downloads/grille-audit-easy-checks.xlsx
+++ b/assets/downloads/grille-audit-easy-checks.xlsx
@@ -7516,7 +7516,7 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>53-55</t>
+          <t>84-86</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>87</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -7612,7 +7612,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>57-58</t>
+          <t>88-89</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -7660,7 +7660,7 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>59-60</t>
+          <t>90-91</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
@@ -7708,7 +7708,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>92</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
@@ -7756,7 +7756,7 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>62-65</t>
+          <t>93-96</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
@@ -7804,7 +7804,7 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>97</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -7852,7 +7852,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>98</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
@@ -7900,7 +7900,7 @@
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>68-69</t>
+          <t>99-100</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
@@ -7948,7 +7948,7 @@
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>101</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
@@ -7996,7 +7996,7 @@
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>102</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
@@ -8044,7 +8044,7 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>72-74</t>
+          <t>105-107</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
@@ -8092,7 +8092,7 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>108</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">

</xml_diff>